<commit_message>
scan: 接力掃描 2026-05-23 11:02 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-05-23.xlsx
+++ b/output/full_scan/batch_seq1_2026-05-23.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CP313"/>
+  <dimension ref="A1:CP322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -89976,6 +89976,2578 @@
       <c r="CO313" t="inlineStr"/>
       <c r="CP313" t="inlineStr"/>
     </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C314" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="D314" t="n">
+        <v>11.05</v>
+      </c>
+      <c r="E314" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="F314" t="n">
+        <v>101107069</v>
+      </c>
+      <c r="G314" t="n">
+        <v>1186348668</v>
+      </c>
+      <c r="H314" t="n">
+        <v>6116</v>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>彩晶</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr"/>
+      <c r="K314" t="n">
+        <v>0.6053998971565235</v>
+      </c>
+      <c r="L314" t="n">
+        <v>0.4334122123385669</v>
+      </c>
+      <c r="M314" t="n">
+        <v>0.1719876848179566</v>
+      </c>
+      <c r="N314" t="n">
+        <v>9.879357469320739</v>
+      </c>
+      <c r="O314" t="n">
+        <v>9.149353871248024</v>
+      </c>
+      <c r="P314" t="n">
+        <v>8.728864348259137</v>
+      </c>
+      <c r="Q314" t="n">
+        <v>71.02638751923888</v>
+      </c>
+      <c r="R314" t="n">
+        <v>35.56102068319223</v>
+      </c>
+      <c r="S314" t="n">
+        <v>0.6326232521189115</v>
+      </c>
+      <c r="T314" t="n">
+        <v>80107191.34999999</v>
+      </c>
+      <c r="U314" t="n">
+        <v>841727012.35</v>
+      </c>
+      <c r="V314" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="W314" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="X314" t="n">
+        <v>1.83614359940066</v>
+      </c>
+      <c r="Y314" t="n">
+        <v>0.2408046891715779</v>
+      </c>
+      <c r="Z314" t="n">
+        <v>0.1560975609756096</v>
+      </c>
+      <c r="AA314" t="n">
+        <v>0.0972222222222221</v>
+      </c>
+      <c r="AB314" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="AC314" t="n">
+        <v>1.136155938187272</v>
+      </c>
+      <c r="AD314" t="n">
+        <v>11.78718327446179</v>
+      </c>
+      <c r="AE314" t="n">
+        <v>9.520000000000016</v>
+      </c>
+      <c r="AF314" t="n">
+        <v>7.252816725538238</v>
+      </c>
+      <c r="AG314" t="n">
+        <v>1.013853473216258</v>
+      </c>
+      <c r="AH314" t="n">
+        <v>0.4762990072398684</v>
+      </c>
+      <c r="AI314" t="n">
+        <v>100</v>
+      </c>
+      <c r="AJ314" t="n">
+        <v>63.94657149037448</v>
+      </c>
+      <c r="AK314" t="n">
+        <v>1188733455</v>
+      </c>
+      <c r="AL314" t="n">
+        <v>806898330.8</v>
+      </c>
+      <c r="AM314" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AN314" t="n">
+        <v>140.1050396692367</v>
+      </c>
+      <c r="AO314" t="n">
+        <v>74.93197231151103</v>
+      </c>
+      <c r="AP314" t="n">
+        <v>8.7575</v>
+      </c>
+      <c r="AQ314" t="n">
+        <v>9.275</v>
+      </c>
+      <c r="AR314" t="n">
+        <v>83262.20116666671</v>
+      </c>
+      <c r="AS314" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT314" t="n">
+        <v>0.0266120113160508</v>
+      </c>
+      <c r="AU314" t="n">
+        <v>24560767</v>
+      </c>
+      <c r="AV314" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW314" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX314" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY314" t="n">
+        <v>745989</v>
+      </c>
+      <c r="AZ314" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA314" t="n">
+        <v>0.1294855496595588</v>
+      </c>
+      <c r="BB314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BE314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BF314" t="n">
+        <v>1.2621472216926</v>
+      </c>
+      <c r="BG314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BJ314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BK314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BM314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BO314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BQ314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BS314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BW314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BX314" t="b">
+        <v>1</v>
+      </c>
+      <c r="BY314" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ314" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA314" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB314" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC314" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CD314" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE314" t="n">
+        <v>13</v>
+      </c>
+      <c r="CF314" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG314" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH314" t="n">
+        <v>1461.131047866074</v>
+      </c>
+      <c r="CI314" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="CJ314" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK314" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL314" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM314" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN314" t="inlineStr">
+        <is>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+        </is>
+      </c>
+      <c r="CO314" t="inlineStr"/>
+      <c r="CP314" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>83.5</v>
+      </c>
+      <c r="C315" t="n">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="D315" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="E315" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="F315" t="n">
+        <v>1400142</v>
+      </c>
+      <c r="G315" t="n">
+        <v>120504601</v>
+      </c>
+      <c r="H315" t="n">
+        <v>6117</v>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>迎廣</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr"/>
+      <c r="K315" t="n">
+        <v>0.6895992304854275</v>
+      </c>
+      <c r="L315" t="n">
+        <v>0.848650082554405</v>
+      </c>
+      <c r="M315" t="n">
+        <v>-0.1590508520689775</v>
+      </c>
+      <c r="N315" t="n">
+        <v>82.35481784113792</v>
+      </c>
+      <c r="O315" t="n">
+        <v>80.00540810179231</v>
+      </c>
+      <c r="P315" t="n">
+        <v>79.91575252151253</v>
+      </c>
+      <c r="Q315" t="n">
+        <v>62.44624491797941</v>
+      </c>
+      <c r="R315" t="n">
+        <v>19.76149663077392</v>
+      </c>
+      <c r="S315" t="n">
+        <v>3.385188505881651</v>
+      </c>
+      <c r="T315" t="n">
+        <v>1117517.45</v>
+      </c>
+      <c r="U315" t="n">
+        <v>96226256.95</v>
+      </c>
+      <c r="V315" t="n">
+        <v>90.7</v>
+      </c>
+      <c r="W315" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="X315" t="n">
+        <v>-0.4858473663935959</v>
+      </c>
+      <c r="Y315" t="n">
+        <v>0.3603271256525664</v>
+      </c>
+      <c r="Z315" t="n">
+        <v>0.0779537149817297</v>
+      </c>
+      <c r="AA315" t="n">
+        <v>0.0714285714285714</v>
+      </c>
+      <c r="AB315" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="AC315" t="n">
+        <v>0.6149986153907016</v>
+      </c>
+      <c r="AD315" t="n">
+        <v>91.70387776812612</v>
+      </c>
+      <c r="AE315" t="n">
+        <v>84.02999999999993</v>
+      </c>
+      <c r="AF315" t="n">
+        <v>76.35612223187373</v>
+      </c>
+      <c r="AG315" t="n">
+        <v>0.7912477977279242</v>
+      </c>
+      <c r="AH315" t="n">
+        <v>0.1826461446656244</v>
+      </c>
+      <c r="AI315" t="n">
+        <v>99.05660377358495</v>
+      </c>
+      <c r="AJ315" t="n">
+        <v>64.68135748175457</v>
+      </c>
+      <c r="AK315" t="n">
+        <v>46723021</v>
+      </c>
+      <c r="AL315" t="n">
+        <v>46790415.45</v>
+      </c>
+      <c r="AM315" t="n">
+        <v>-4.545454545454546</v>
+      </c>
+      <c r="AN315" t="n">
+        <v>47.19736222326913</v>
+      </c>
+      <c r="AO315" t="n">
+        <v>40.63540525765376</v>
+      </c>
+      <c r="AP315" t="n">
+        <v>74.69999999999999</v>
+      </c>
+      <c r="AQ315" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="AR315" t="n">
+        <v>83262.20116666671</v>
+      </c>
+      <c r="AS315" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT315" t="n">
+        <v>0.0266120113160508</v>
+      </c>
+      <c r="AU315" t="n">
+        <v>541000</v>
+      </c>
+      <c r="AV315" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW315" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX315" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY315" t="n">
+        <v>37000</v>
+      </c>
+      <c r="AZ315" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA315" t="n">
+        <v>0.0513417036656789</v>
+      </c>
+      <c r="BB315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD315" t="b">
+        <v>1</v>
+      </c>
+      <c r="BE315" t="b">
+        <v>1</v>
+      </c>
+      <c r="BF315" t="n">
+        <v>1.252903925571811</v>
+      </c>
+      <c r="BG315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH315" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL315" t="b">
+        <v>1</v>
+      </c>
+      <c r="BM315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN315" t="b">
+        <v>1</v>
+      </c>
+      <c r="BO315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BX315" t="b">
+        <v>1</v>
+      </c>
+      <c r="BY315" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ315" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA315" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB315" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC315" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CD315" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE315" t="n">
+        <v>7</v>
+      </c>
+      <c r="CF315" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG315" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH315" t="n">
+        <v>767.4247062530599</v>
+      </c>
+      <c r="CI315" t="n">
+        <v>26</v>
+      </c>
+      <c r="CJ315" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK315" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL315" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM315" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN315" t="inlineStr">
+        <is>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, stronger_than_market, above_ichimoku_cloud</t>
+        </is>
+      </c>
+      <c r="CO315" t="inlineStr"/>
+      <c r="CP315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="C316" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D316" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="E316" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="F316" t="n">
+        <v>13984511</v>
+      </c>
+      <c r="G316" t="n">
+        <v>202973457</v>
+      </c>
+      <c r="H316" t="n">
+        <v>6120</v>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>達運</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr"/>
+      <c r="K316" t="n">
+        <v>-0.0221645973668316</v>
+      </c>
+      <c r="L316" t="n">
+        <v>-0.152608052825178</v>
+      </c>
+      <c r="M316" t="n">
+        <v>0.1304434554583464</v>
+      </c>
+      <c r="N316" t="n">
+        <v>13.25760742027481</v>
+      </c>
+      <c r="O316" t="n">
+        <v>13.24402776450482</v>
+      </c>
+      <c r="P316" t="n">
+        <v>12.90952179121286</v>
+      </c>
+      <c r="Q316" t="n">
+        <v>65.57815576875859</v>
+      </c>
+      <c r="R316" t="n">
+        <v>13.11818373735263</v>
+      </c>
+      <c r="S316" t="n">
+        <v>0.6512103120711608</v>
+      </c>
+      <c r="T316" t="n">
+        <v>3835241.5</v>
+      </c>
+      <c r="U316" t="n">
+        <v>50925065.65</v>
+      </c>
+      <c r="V316" t="n">
+        <v>13.45</v>
+      </c>
+      <c r="W316" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="X316" t="n">
+        <v>0.0877937659875295</v>
+      </c>
+      <c r="Y316" t="n">
+        <v>0.0141405925645264</v>
+      </c>
+      <c r="Z316" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="AA316" t="n">
+        <v>0.09701492537313421</v>
+      </c>
+      <c r="AB316" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="AC316" t="n">
+        <v>1.6842357689339</v>
+      </c>
+      <c r="AD316" t="n">
+        <v>13.96561090377242</v>
+      </c>
+      <c r="AE316" t="n">
+        <v>13.06500000000001</v>
+      </c>
+      <c r="AF316" t="n">
+        <v>12.1643890962276</v>
+      </c>
+      <c r="AG316" t="n">
+        <v>1.40771719127063</v>
+      </c>
+      <c r="AH316" t="n">
+        <v>0.1378661926938246</v>
+      </c>
+      <c r="AI316" t="n">
+        <v>100</v>
+      </c>
+      <c r="AJ316" t="n">
+        <v>77.33333333333333</v>
+      </c>
+      <c r="AK316" t="n">
+        <v>118768688</v>
+      </c>
+      <c r="AL316" t="n">
+        <v>102006825.75</v>
+      </c>
+      <c r="AM316" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AN316" t="n">
+        <v>336.1227336122752</v>
+      </c>
+      <c r="AO316" t="n">
+        <v>69.75720523764682</v>
+      </c>
+      <c r="AP316" t="n">
+        <v>13.875</v>
+      </c>
+      <c r="AQ316" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="AR316" t="n">
+        <v>83262.20116666671</v>
+      </c>
+      <c r="AS316" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT316" t="n">
+        <v>0.0266120113160508</v>
+      </c>
+      <c r="AU316" t="n">
+        <v>6592760</v>
+      </c>
+      <c r="AV316" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW316" t="n">
+        <v>84000</v>
+      </c>
+      <c r="AX316" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY316" t="n">
+        <v>519783</v>
+      </c>
+      <c r="AZ316" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA316" t="n">
+        <v>0.1400546553506159</v>
+      </c>
+      <c r="BB316" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC316" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BE316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BF316" t="n">
+        <v>3.64631823054689</v>
+      </c>
+      <c r="BG316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI316" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BK316" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BM316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BN316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BO316" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BQ316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BR316" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BT316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BU316" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BW316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BX316" t="b">
+        <v>1</v>
+      </c>
+      <c r="BY316" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ316" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA316" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB316" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC316" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CD316" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE316" t="n">
+        <v>16</v>
+      </c>
+      <c r="CF316" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG316" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH316" t="n">
+        <v>1848.586831577883</v>
+      </c>
+      <c r="CI316" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="CJ316" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK316" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL316" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM316" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN316" t="inlineStr">
+        <is>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, invest_trust_buy_2d, bb_squeeze_breakout, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+        </is>
+      </c>
+      <c r="CO316" t="inlineStr"/>
+      <c r="CP316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>47.05</v>
+      </c>
+      <c r="C317" t="n">
+        <v>47.05</v>
+      </c>
+      <c r="D317" t="n">
+        <v>46.75</v>
+      </c>
+      <c r="E317" t="n">
+        <v>46.95</v>
+      </c>
+      <c r="F317" t="n">
+        <v>142540</v>
+      </c>
+      <c r="G317" t="n">
+        <v>6683680</v>
+      </c>
+      <c r="H317" t="n">
+        <v>6115</v>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>鎰勝</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr"/>
+      <c r="K317" t="n">
+        <v>-0.1594618924258881</v>
+      </c>
+      <c r="L317" t="n">
+        <v>-0.0712096543595125</v>
+      </c>
+      <c r="M317" t="n">
+        <v>-0.0882522380663756</v>
+      </c>
+      <c r="N317" t="n">
+        <v>47.23317616514879</v>
+      </c>
+      <c r="O317" t="n">
+        <v>47.25973401462687</v>
+      </c>
+      <c r="P317" t="n">
+        <v>47.34506792246505</v>
+      </c>
+      <c r="Q317" t="n">
+        <v>42.19063856340242</v>
+      </c>
+      <c r="R317" t="n">
+        <v>17.34245146671823</v>
+      </c>
+      <c r="S317" t="n">
+        <v>0.4128703418057111</v>
+      </c>
+      <c r="T317" t="n">
+        <v>184804.05</v>
+      </c>
+      <c r="U317" t="n">
+        <v>8769611</v>
+      </c>
+      <c r="V317" t="n">
+        <v>48.15</v>
+      </c>
+      <c r="W317" t="n">
+        <v>46.65</v>
+      </c>
+      <c r="X317" t="n">
+        <v>-0.1403143168710429</v>
+      </c>
+      <c r="Y317" t="n">
+        <v>0.0128482155458562</v>
+      </c>
+      <c r="Z317" t="n">
+        <v>0.0053533190578158</v>
+      </c>
+      <c r="AA317" t="n">
+        <v>-0.0010638297872339</v>
+      </c>
+      <c r="AB317" t="n">
+        <v>47</v>
+      </c>
+      <c r="AC317" t="n">
+        <v>0.3617519911780532</v>
+      </c>
+      <c r="AD317" t="n">
+        <v>48.31741712328948</v>
+      </c>
+      <c r="AE317" t="n">
+        <v>47.41249999999991</v>
+      </c>
+      <c r="AF317" t="n">
+        <v>46.50758287671034</v>
+      </c>
+      <c r="AG317" t="n">
+        <v>0.244451735912225</v>
+      </c>
+      <c r="AH317" t="n">
+        <v>0.0381720906212316</v>
+      </c>
+      <c r="AI317" t="n">
+        <v>42.3076923076925</v>
+      </c>
+      <c r="AJ317" t="n">
+        <v>36.95970695970694</v>
+      </c>
+      <c r="AK317" t="n">
+        <v>-3028126</v>
+      </c>
+      <c r="AL317" t="n">
+        <v>-2376012.5</v>
+      </c>
+      <c r="AM317" t="n">
+        <v>-68.57142857142833</v>
+      </c>
+      <c r="AN317" t="n">
+        <v>-83.68084514873622</v>
+      </c>
+      <c r="AO317" t="n">
+        <v>52.62417759813473</v>
+      </c>
+      <c r="AP317" t="n">
+        <v>47</v>
+      </c>
+      <c r="AQ317" t="n">
+        <v>47.075</v>
+      </c>
+      <c r="AR317" t="n">
+        <v>83262.20116666671</v>
+      </c>
+      <c r="AS317" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT317" t="n">
+        <v>0.0266120113160508</v>
+      </c>
+      <c r="AU317" t="n">
+        <v>-78000</v>
+      </c>
+      <c r="AV317" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW317" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX317" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY317" t="n">
+        <v>-358</v>
+      </c>
+      <c r="AZ317" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA317" t="n">
+        <v>-0.0212586922582349</v>
+      </c>
+      <c r="BB317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BE317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF317" t="n">
+        <v>0.7713034427546367</v>
+      </c>
+      <c r="BG317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BI317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK317" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BO317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW317" t="b">
+        <v>1</v>
+      </c>
+      <c r="BX317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY317" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ317" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA317" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB317" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC317" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CD317" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE317" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF317" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG317" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH317" t="n">
+        <v>332.929616668441</v>
+      </c>
+      <c r="CI317" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="CJ317" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK317" t="b">
+        <v>1</v>
+      </c>
+      <c r="CL317" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM317" t="b">
+        <v>1</v>
+      </c>
+      <c r="CN317" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+        </is>
+      </c>
+      <c r="CO317" t="inlineStr"/>
+      <c r="CP317" t="inlineStr">
+        <is>
+          <t>close_below_ema20</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B318" t="n">
+        <v>18.95</v>
+      </c>
+      <c r="C318" t="n">
+        <v>19.05</v>
+      </c>
+      <c r="D318" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="E318" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="F318" t="n">
+        <v>377247</v>
+      </c>
+      <c r="G318" t="n">
+        <v>7107211</v>
+      </c>
+      <c r="H318" t="n">
+        <v>6128</v>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>上福</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr"/>
+      <c r="K318" t="n">
+        <v>-0.601117283923255</v>
+      </c>
+      <c r="L318" t="n">
+        <v>-0.506240016010775</v>
+      </c>
+      <c r="M318" t="n">
+        <v>-0.09487726791248</v>
+      </c>
+      <c r="N318" t="n">
+        <v>19.87161583190396</v>
+      </c>
+      <c r="O318" t="n">
+        <v>21.16523854065663</v>
+      </c>
+      <c r="P318" t="n">
+        <v>22.67586904219697</v>
+      </c>
+      <c r="Q318" t="n">
+        <v>29.64413074593791</v>
+      </c>
+      <c r="R318" t="n">
+        <v>28.55620988870711</v>
+      </c>
+      <c r="S318" t="n">
+        <v>0.3971415862532879</v>
+      </c>
+      <c r="T318" t="n">
+        <v>155590.85</v>
+      </c>
+      <c r="U318" t="n">
+        <v>3098046.2</v>
+      </c>
+      <c r="V318" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="W318" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="X318" t="n">
+        <v>-0.5455058990336736</v>
+      </c>
+      <c r="Y318" t="n">
+        <v>-0.4323356449870408</v>
+      </c>
+      <c r="Z318" t="n">
+        <v>-0.0284237726098192</v>
+      </c>
+      <c r="AA318" t="n">
+        <v>-0.0208333333333332</v>
+      </c>
+      <c r="AB318" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="AC318" t="n">
+        <v>1.294592193914032</v>
+      </c>
+      <c r="AD318" t="n">
+        <v>21.43442158912621</v>
+      </c>
+      <c r="AE318" t="n">
+        <v>20.03000000000002</v>
+      </c>
+      <c r="AF318" t="n">
+        <v>18.62557841087382</v>
+      </c>
+      <c r="AG318" t="n">
+        <v>0.0620973041416637</v>
+      </c>
+      <c r="AH318" t="n">
+        <v>0.1402318111958255</v>
+      </c>
+      <c r="AI318" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ318" t="n">
+        <v>7.619047619047706</v>
+      </c>
+      <c r="AK318" t="n">
+        <v>-9242586</v>
+      </c>
+      <c r="AL318" t="n">
+        <v>-8510114.449999999</v>
+      </c>
+      <c r="AM318" t="n">
+        <v>-100</v>
+      </c>
+      <c r="AN318" t="n">
+        <v>-131.646755680487</v>
+      </c>
+      <c r="AO318" t="n">
+        <v>30.68535828455378</v>
+      </c>
+      <c r="AP318" t="n">
+        <v>21.6625</v>
+      </c>
+      <c r="AQ318" t="n">
+        <v>23.925</v>
+      </c>
+      <c r="AR318" t="n">
+        <v>83262.20116666671</v>
+      </c>
+      <c r="AS318" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT318" t="n">
+        <v>0.0266120113160508</v>
+      </c>
+      <c r="AU318" t="n">
+        <v>36000</v>
+      </c>
+      <c r="AV318" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW318" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX318" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY318" t="n">
+        <v>-295</v>
+      </c>
+      <c r="AZ318" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA318" t="n">
+        <v>-0.05503578392587</v>
+      </c>
+      <c r="BB318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BE318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF318" t="n">
+        <v>2.424609159214697</v>
+      </c>
+      <c r="BG318" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BI318" t="b">
+        <v>1</v>
+      </c>
+      <c r="BJ318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK318" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BO318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BX318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY318" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ318" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA318" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB318" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC318" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CD318" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE318" t="n">
+        <v>4</v>
+      </c>
+      <c r="CF318" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG318" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH318" t="n">
+        <v>462.298723088267</v>
+      </c>
+      <c r="CI318" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="CJ318" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK318" t="b">
+        <v>1</v>
+      </c>
+      <c r="CL318" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM318" t="b">
+        <v>1</v>
+      </c>
+      <c r="CN318" t="inlineStr">
+        <is>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+        </is>
+      </c>
+      <c r="CO318" t="inlineStr"/>
+      <c r="CP318" t="inlineStr">
+        <is>
+          <t>close_below_ema20</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B319" t="n">
+        <v>24</v>
+      </c>
+      <c r="C319" t="n">
+        <v>24.25</v>
+      </c>
+      <c r="D319" t="n">
+        <v>23.65</v>
+      </c>
+      <c r="E319" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="F319" t="n">
+        <v>2771330</v>
+      </c>
+      <c r="G319" t="n">
+        <v>66499641</v>
+      </c>
+      <c r="H319" t="n">
+        <v>6133</v>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>金橋</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr"/>
+      <c r="K319" t="n">
+        <v>0.1331011835465538</v>
+      </c>
+      <c r="L319" t="n">
+        <v>-0.1825613498803475</v>
+      </c>
+      <c r="M319" t="n">
+        <v>0.3156625334269014</v>
+      </c>
+      <c r="N319" t="n">
+        <v>22.59416602580929</v>
+      </c>
+      <c r="O319" t="n">
+        <v>22.6568125621494</v>
+      </c>
+      <c r="P319" t="n">
+        <v>21.82031763653869</v>
+      </c>
+      <c r="Q319" t="n">
+        <v>60.5603661989443</v>
+      </c>
+      <c r="R319" t="n">
+        <v>12.12654814370055</v>
+      </c>
+      <c r="S319" t="n">
+        <v>0.9899337550387892</v>
+      </c>
+      <c r="T319" t="n">
+        <v>1813882.45</v>
+      </c>
+      <c r="U319" t="n">
+        <v>41931261.6</v>
+      </c>
+      <c r="V319" t="n">
+        <v>24.35</v>
+      </c>
+      <c r="W319" t="n">
+        <v>20.55</v>
+      </c>
+      <c r="X319" t="n">
+        <v>0.3074573964755623</v>
+      </c>
+      <c r="Y319" t="n">
+        <v>-0.2197762386934294</v>
+      </c>
+      <c r="Z319" t="n">
+        <v>0.1476190476190477</v>
+      </c>
+      <c r="AA319" t="n">
+        <v>0.0041666666666666</v>
+      </c>
+      <c r="AB319" t="n">
+        <v>24</v>
+      </c>
+      <c r="AC319" t="n">
+        <v>2.423612894891404</v>
+      </c>
+      <c r="AD319" t="n">
+        <v>24.13902716804128</v>
+      </c>
+      <c r="AE319" t="n">
+        <v>22.225</v>
+      </c>
+      <c r="AF319" t="n">
+        <v>20.31097283195873</v>
+      </c>
+      <c r="AG319" t="n">
+        <v>0.989804959748504</v>
+      </c>
+      <c r="AH319" t="n">
+        <v>0.1722409150093386</v>
+      </c>
+      <c r="AI319" t="n">
+        <v>86.20689655172418</v>
+      </c>
+      <c r="AJ319" t="n">
+        <v>88.45101258894404</v>
+      </c>
+      <c r="AK319" t="n">
+        <v>113123480</v>
+      </c>
+      <c r="AL319" t="n">
+        <v>104771249.4</v>
+      </c>
+      <c r="AM319" t="n">
+        <v>-13.79310344827582</v>
+      </c>
+      <c r="AN319" t="n">
+        <v>178.5198402583049</v>
+      </c>
+      <c r="AO319" t="n">
+        <v>57.94033430666515</v>
+      </c>
+      <c r="AP319" t="n">
+        <v>23.9875</v>
+      </c>
+      <c r="AQ319" t="n">
+        <v>25.55</v>
+      </c>
+      <c r="AR319" t="n">
+        <v>83262.20116666671</v>
+      </c>
+      <c r="AS319" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT319" t="n">
+        <v>0.0266120113160508</v>
+      </c>
+      <c r="AU319" t="n">
+        <v>80000</v>
+      </c>
+      <c r="AV319" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW319" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX319" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY319" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ319" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA319" t="n">
+        <v>0.1210070363029969</v>
+      </c>
+      <c r="BB319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD319" t="b">
+        <v>1</v>
+      </c>
+      <c r="BE319" t="b">
+        <v>1</v>
+      </c>
+      <c r="BF319" t="n">
+        <v>1.527844320893011</v>
+      </c>
+      <c r="BG319" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH319" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN319" t="b">
+        <v>1</v>
+      </c>
+      <c r="BO319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP319" t="b">
+        <v>1</v>
+      </c>
+      <c r="BQ319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW319" t="b">
+        <v>1</v>
+      </c>
+      <c r="BX319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY319" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ319" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA319" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB319" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC319" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CD319" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE319" t="n">
+        <v>8</v>
+      </c>
+      <c r="CF319" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG319" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH319" t="n">
+        <v>874.5056949829303</v>
+      </c>
+      <c r="CI319" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="CJ319" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK319" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL319" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM319" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN319" t="inlineStr">
+        <is>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong</t>
+        </is>
+      </c>
+      <c r="CO319" t="inlineStr"/>
+      <c r="CP319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B320" t="n">
+        <v>808</v>
+      </c>
+      <c r="C320" t="n">
+        <v>808</v>
+      </c>
+      <c r="D320" t="n">
+        <v>767</v>
+      </c>
+      <c r="E320" t="n">
+        <v>769</v>
+      </c>
+      <c r="F320" t="n">
+        <v>6471356</v>
+      </c>
+      <c r="G320" t="n">
+        <v>5075673886</v>
+      </c>
+      <c r="H320" t="n">
+        <v>6139</v>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>亞翔</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr"/>
+      <c r="K320" t="n">
+        <v>28.59967006801605</v>
+      </c>
+      <c r="L320" t="n">
+        <v>24.85475648934434</v>
+      </c>
+      <c r="M320" t="n">
+        <v>3.744913578671706</v>
+      </c>
+      <c r="N320" t="n">
+        <v>709.3366174910659</v>
+      </c>
+      <c r="O320" t="n">
+        <v>647.3601972080713</v>
+      </c>
+      <c r="P320" t="n">
+        <v>585.4079340341264</v>
+      </c>
+      <c r="Q320" t="n">
+        <v>62.98820292714004</v>
+      </c>
+      <c r="R320" t="n">
+        <v>22.58192627934615</v>
+      </c>
+      <c r="S320" t="n">
+        <v>43.54291217768997</v>
+      </c>
+      <c r="T320" t="n">
+        <v>4764499.7</v>
+      </c>
+      <c r="U320" t="n">
+        <v>3406764543.3</v>
+      </c>
+      <c r="V320" t="n">
+        <v>784</v>
+      </c>
+      <c r="W320" t="n">
+        <v>679</v>
+      </c>
+      <c r="X320" t="n">
+        <v>0.5359104021561616</v>
+      </c>
+      <c r="Y320" t="n">
+        <v>0.6387549563000577</v>
+      </c>
+      <c r="Z320" t="n">
+        <v>0.1096681096681095</v>
+      </c>
+      <c r="AA320" t="n">
+        <v>-0.0191326530612244</v>
+      </c>
+      <c r="AB320" t="n">
+        <v>784</v>
+      </c>
+      <c r="AC320" t="n">
+        <v>1.642641087392265</v>
+      </c>
+      <c r="AD320" t="n">
+        <v>767.8869841048119</v>
+      </c>
+      <c r="AE320" t="n">
+        <v>705.95</v>
+      </c>
+      <c r="AF320" t="n">
+        <v>644.0130158951882</v>
+      </c>
+      <c r="AG320" t="n">
+        <v>1.008985066929516</v>
+      </c>
+      <c r="AH320" t="n">
+        <v>0.1754713056301772</v>
+      </c>
+      <c r="AI320" t="n">
+        <v>73.10344827586206</v>
+      </c>
+      <c r="AJ320" t="n">
+        <v>75.39370924174061</v>
+      </c>
+      <c r="AK320" t="n">
+        <v>395043675</v>
+      </c>
+      <c r="AL320" t="n">
+        <v>388239662.85</v>
+      </c>
+      <c r="AM320" t="n">
+        <v>-25.49019607843137</v>
+      </c>
+      <c r="AN320" t="n">
+        <v>213.5289323553378</v>
+      </c>
+      <c r="AO320" t="n">
+        <v>60.18119326130424</v>
+      </c>
+      <c r="AP320" t="n">
+        <v>581.125</v>
+      </c>
+      <c r="AQ320" t="n">
+        <v>574.75</v>
+      </c>
+      <c r="AR320" t="n">
+        <v>83262.20116666671</v>
+      </c>
+      <c r="AS320" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT320" t="n">
+        <v>0.0266120113160508</v>
+      </c>
+      <c r="AU320" t="n">
+        <v>-2102139</v>
+      </c>
+      <c r="AV320" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW320" t="n">
+        <v>1043000</v>
+      </c>
+      <c r="AX320" t="n">
+        <v>8</v>
+      </c>
+      <c r="AY320" t="n">
+        <v>-121487</v>
+      </c>
+      <c r="AZ320" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA320" t="n">
+        <v>0.0830560983520587</v>
+      </c>
+      <c r="BB320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BE320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BF320" t="n">
+        <v>1.358244602261178</v>
+      </c>
+      <c r="BG320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BJ320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BM320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BO320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BQ320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BR320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BT320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BX320" t="b">
+        <v>1</v>
+      </c>
+      <c r="BY320" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ320" t="b">
+        <v>1</v>
+      </c>
+      <c r="CA320" t="b">
+        <v>1</v>
+      </c>
+      <c r="CB320" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC320" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CD320" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE320" t="n">
+        <v>12</v>
+      </c>
+      <c r="CF320" t="b">
+        <v>1</v>
+      </c>
+      <c r="CG320" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH320" t="n">
+        <v>1379.469982137164</v>
+      </c>
+      <c r="CI320" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="CJ320" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK320" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL320" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM320" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN320" t="inlineStr">
+        <is>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
+        </is>
+      </c>
+      <c r="CO320" t="inlineStr">
+        <is>
+          <t>open_high_close_low, gap_chase_after_blowout</t>
+        </is>
+      </c>
+      <c r="CP320" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B321" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="C321" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="D321" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="E321" t="n">
+        <v>34</v>
+      </c>
+      <c r="F321" t="n">
+        <v>2552418</v>
+      </c>
+      <c r="G321" t="n">
+        <v>88636589</v>
+      </c>
+      <c r="H321" t="n">
+        <v>6141</v>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>柏承</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr"/>
+      <c r="K321" t="n">
+        <v>1.506118809469907</v>
+      </c>
+      <c r="L321" t="n">
+        <v>1.694593161082123</v>
+      </c>
+      <c r="M321" t="n">
+        <v>-0.1884743516122164</v>
+      </c>
+      <c r="N321" t="n">
+        <v>31.69556206832608</v>
+      </c>
+      <c r="O321" t="n">
+        <v>26.37239465464055</v>
+      </c>
+      <c r="P321" t="n">
+        <v>21.46076682572066</v>
+      </c>
+      <c r="Q321" t="n">
+        <v>58.07284773399088</v>
+      </c>
+      <c r="R321" t="n">
+        <v>23.69783336511352</v>
+      </c>
+      <c r="S321" t="n">
+        <v>2.92194227705927</v>
+      </c>
+      <c r="T321" t="n">
+        <v>2182305.25</v>
+      </c>
+      <c r="U321" t="n">
+        <v>70386943.25</v>
+      </c>
+      <c r="V321" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="W321" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="X321" t="n">
+        <v>-0.0563658261712555</v>
+      </c>
+      <c r="Y321" t="n">
+        <v>1.528595705823293</v>
+      </c>
+      <c r="Z321" t="n">
+        <v>0.2035398230088496</v>
+      </c>
+      <c r="AA321" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB321" t="n">
+        <v>34</v>
+      </c>
+      <c r="AC321" t="n">
+        <v>1.588334189142588</v>
+      </c>
+      <c r="AD321" t="n">
+        <v>38.00060992991237</v>
+      </c>
+      <c r="AE321" t="n">
+        <v>32.49249999999999</v>
+      </c>
+      <c r="AF321" t="n">
+        <v>26.98439007008761</v>
+      </c>
+      <c r="AG321" t="n">
+        <v>0.6368436740716963</v>
+      </c>
+      <c r="AH321" t="n">
+        <v>0.3390388508063325</v>
+      </c>
+      <c r="AI321" t="n">
+        <v>76.678445229682</v>
+      </c>
+      <c r="AJ321" t="n">
+        <v>77.85630153121262</v>
+      </c>
+      <c r="AK321" t="n">
+        <v>91575515</v>
+      </c>
+      <c r="AL321" t="n">
+        <v>80622123.5</v>
+      </c>
+      <c r="AM321" t="n">
+        <v>-31.54574132492113</v>
+      </c>
+      <c r="AN321" t="n">
+        <v>59.85149451381008</v>
+      </c>
+      <c r="AO321" t="n">
+        <v>67.96079872921476</v>
+      </c>
+      <c r="AP321" t="n">
+        <v>22.55</v>
+      </c>
+      <c r="AQ321" t="n">
+        <v>19.525</v>
+      </c>
+      <c r="AR321" t="n">
+        <v>83262.20116666671</v>
+      </c>
+      <c r="AS321" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT321" t="n">
+        <v>0.0266120113160508</v>
+      </c>
+      <c r="AU321" t="n">
+        <v>-38000</v>
+      </c>
+      <c r="AV321" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW321" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX321" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY321" t="n">
+        <v>-17000</v>
+      </c>
+      <c r="AZ321" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA321" t="n">
+        <v>0.1769278116927988</v>
+      </c>
+      <c r="BB321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD321" t="b">
+        <v>1</v>
+      </c>
+      <c r="BE321" t="b">
+        <v>1</v>
+      </c>
+      <c r="BF321" t="n">
+        <v>1.169597149619651</v>
+      </c>
+      <c r="BG321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH321" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI321" t="b">
+        <v>1</v>
+      </c>
+      <c r="BJ321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL321" t="b">
+        <v>1</v>
+      </c>
+      <c r="BM321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN321" t="b">
+        <v>1</v>
+      </c>
+      <c r="BO321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP321" t="b">
+        <v>1</v>
+      </c>
+      <c r="BQ321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV321" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW321" t="b">
+        <v>1</v>
+      </c>
+      <c r="BX321" t="b">
+        <v>1</v>
+      </c>
+      <c r="BY321" t="b">
+        <v>1</v>
+      </c>
+      <c r="BZ321" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA321" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB321" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC321" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CD321" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE321" t="n">
+        <v>10</v>
+      </c>
+      <c r="CF321" t="b">
+        <v>1</v>
+      </c>
+      <c r="CG321" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH321" t="n">
+        <v>1123.08658603059</v>
+      </c>
+      <c r="CI321" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="CJ321" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK321" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL321" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM321" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN321" t="inlineStr">
+        <is>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+        </is>
+      </c>
+      <c r="CO321" t="inlineStr">
+        <is>
+          <t>long_upper_shadow</t>
+        </is>
+      </c>
+      <c r="CP321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>25.45</v>
+      </c>
+      <c r="C322" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="D322" t="n">
+        <v>25.05</v>
+      </c>
+      <c r="E322" t="n">
+        <v>25.75</v>
+      </c>
+      <c r="F322" t="n">
+        <v>568045</v>
+      </c>
+      <c r="G322" t="n">
+        <v>14485152</v>
+      </c>
+      <c r="H322" t="n">
+        <v>6136</v>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>富爾特</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr"/>
+      <c r="K322" t="n">
+        <v>0.0492732336010881</v>
+      </c>
+      <c r="L322" t="n">
+        <v>0.0607885246583408</v>
+      </c>
+      <c r="M322" t="n">
+        <v>-0.0115152910572526</v>
+      </c>
+      <c r="N322" t="n">
+        <v>25.22067846291198</v>
+      </c>
+      <c r="O322" t="n">
+        <v>24.85930958733829</v>
+      </c>
+      <c r="P322" t="n">
+        <v>24.47930461007507</v>
+      </c>
+      <c r="Q322" t="n">
+        <v>56.03377802514607</v>
+      </c>
+      <c r="R322" t="n">
+        <v>15.05956115026762</v>
+      </c>
+      <c r="S322" t="n">
+        <v>0.6912435090640938</v>
+      </c>
+      <c r="T322" t="n">
+        <v>733963</v>
+      </c>
+      <c r="U322" t="n">
+        <v>19119666.75</v>
+      </c>
+      <c r="V322" t="n">
+        <v>28</v>
+      </c>
+      <c r="W322" t="n">
+        <v>24.55</v>
+      </c>
+      <c r="X322" t="n">
+        <v>-0.2186406837013886</v>
+      </c>
+      <c r="Y322" t="n">
+        <v>0.1431755196808857</v>
+      </c>
+      <c r="Z322" t="n">
+        <v>0.0362173038229376</v>
+      </c>
+      <c r="AA322" t="n">
+        <v>0.0117878192534381</v>
+      </c>
+      <c r="AB322" t="n">
+        <v>25.45</v>
+      </c>
+      <c r="AC322" t="n">
+        <v>0.4282715054257472</v>
+      </c>
+      <c r="AD322" t="n">
+        <v>26.81361641018301</v>
+      </c>
+      <c r="AE322" t="n">
+        <v>25.35749999999998</v>
+      </c>
+      <c r="AF322" t="n">
+        <v>23.90138358981695</v>
+      </c>
+      <c r="AG322" t="n">
+        <v>0.6347763122698012</v>
+      </c>
+      <c r="AH322" t="n">
+        <v>0.114847000704567</v>
+      </c>
+      <c r="AI322" t="n">
+        <v>96.1538461538461</v>
+      </c>
+      <c r="AJ322" t="n">
+        <v>64.37451437451455</v>
+      </c>
+      <c r="AK322" t="n">
+        <v>6976634</v>
+      </c>
+      <c r="AL322" t="n">
+        <v>6934038.45</v>
+      </c>
+      <c r="AM322" t="n">
+        <v>-23.52941176470581</v>
+      </c>
+      <c r="AN322" t="n">
+        <v>15.53004726536152</v>
+      </c>
+      <c r="AO322" t="n">
+        <v>52.18075905069001</v>
+      </c>
+      <c r="AP322" t="n">
+        <v>24.25</v>
+      </c>
+      <c r="AQ322" t="n">
+        <v>24.15</v>
+      </c>
+      <c r="AR322" t="n">
+        <v>83262.20116666671</v>
+      </c>
+      <c r="AS322" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT322" t="n">
+        <v>0.0266120113160508</v>
+      </c>
+      <c r="AU322" t="n">
+        <v>21000</v>
+      </c>
+      <c r="AV322" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW322" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX322" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY322" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ322" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA322" t="n">
+        <v>0.009605292506886701</v>
+      </c>
+      <c r="BB322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD322" t="b">
+        <v>1</v>
+      </c>
+      <c r="BE322" t="b">
+        <v>1</v>
+      </c>
+      <c r="BF322" t="n">
+        <v>0.773942283194112</v>
+      </c>
+      <c r="BG322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH322" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK322" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM322" t="b">
+        <v>1</v>
+      </c>
+      <c r="BN322" t="b">
+        <v>1</v>
+      </c>
+      <c r="BO322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP322" t="b">
+        <v>1</v>
+      </c>
+      <c r="BQ322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW322" t="b">
+        <v>1</v>
+      </c>
+      <c r="BX322" t="b">
+        <v>1</v>
+      </c>
+      <c r="BY322" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ322" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA322" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB322" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC322" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CD322" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE322" t="n">
+        <v>10</v>
+      </c>
+      <c r="CF322" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG322" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH322" t="n">
+        <v>1108.759513232898</v>
+      </c>
+      <c r="CI322" t="n">
+        <v>13</v>
+      </c>
+      <c r="CJ322" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK322" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL322" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM322" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN322" t="inlineStr">
+        <is>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+        </is>
+      </c>
+      <c r="CO322" t="inlineStr"/>
+      <c r="CP322" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>